<commit_message>
fix(prototype): catch a postcode that sits outside its state
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcN31rp9VbcJRWXbFJQ4Vv
</commit_message>
<xml_diff>
--- a/public/sample-data/au-audience-consented.xlsx
+++ b/public/sample-data/au-audience-consented.xlsx
@@ -17009,7 +17009,7 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>302</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -20486,7 +20486,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>(07) 5550 5647</t>
+          <t>(03) 5550 4417</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
@@ -20499,27 +20499,27 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>QLD</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>Sunnybank</t>
+          <t>Tarneit</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>4109</t>
+          <t>2150</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>303061080</t>
+          <t>213051588</t>
         </is>
       </c>
       <c r="L201" t="inlineStr">
         <is>
-          <t>Sunnybank Hills</t>
+          <t>Truganina - South West</t>
         </is>
       </c>
       <c r="M201" t="inlineStr">

</xml_diff>